<commit_message>
Phase 5 done: Prowler #3 (CIS 67.71%), sanitized summary, register + README updated
</commit_message>
<xml_diff>
--- a/reports/risk-register.xlsx
+++ b/reports/risk-register.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="227">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -123,180 +123,183 @@
     <t xml:space="preserve">Mitigate</t>
   </si>
   <si>
-    <t xml:space="preserve">Account-level S3 BPA; L1 also removes public policy statement</t>
+    <t xml:space="preserve">Account-level S3 BPA (done 2026-10-25, CIS 3.1.4 pass); L1 should also remove the public policy statement</t>
   </si>
   <si>
     <t xml:space="preserve">Ziad A.</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.15, 5.23, 8.3, 8.12, 8.24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 Storage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long-lived CI access key leaked through source code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev-ci IAM user, data bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">External attacker / secret-scanning bots</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Static key stored in a file in Git history; no secret scanning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Least-privilege dev-ci (no kms:Decrypt); Wazuh 100110 (unknown IP); RB-S2 runbook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detected 3 min 41 s after first misuse; contained 2 min 42 s after alert; KMS copy denied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OIDC federation for CI (no standing keys); pre-commit + push-protection secret scanning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recommended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.17, 8.4, 8.5, 8.28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 IAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attacker persistence through additional access keys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAM users</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attacker holding a valid key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identity allowed to create its own keys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wazuh 100113 (level 14) via us-east-1 IAM poller; AWSDenyAll-first containment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Persistence detected 3 min 40 s after creation; neutralized 5 min 21 s after creation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove iam:CreateAccessKey from CI identities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.16, 5.18, 8.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administrative port exposed to the internet and attacked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EC2 web instance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internet scanners, brute force</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security group can be opened to 0.0.0.0/0; no NACL second layer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No key pair, no password auth, SSM only; Wazuh 100121 + 5710/5712; Lambda L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hydra aborted (no password auth); S3a manual 7 min 57 s; S3b L2 5.3 s; agent detection in seconds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NACL + VPC flow logs done 2026-10-25 (CIS 4.7 pass); 100121+57xx correlation recommended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.20, 8.22, 8.5, 8.16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 Networking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instance role credentials stolen through IMDSv1 + SSRF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M-IMDS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lab-web-role credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attacker exploiting a web SSRF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMDSv1 can be re-enabled per instance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMDSv2 required, hop limit 1; Lambda L3; Wazuh 100132; rules 100130/131/133 for credential use outside the instance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L3 fixed in 6.4 s; 100132 in 1 min 23 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account default IMDSv2 required (done 2026-10-25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.9, 8.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automated remediation silently not working</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1b-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lambda L1-L3 / EventBridge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operational failure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rule changes and new trails are eventually consistent; no health check of automation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIEM detection independent of automation; session checklist (wait ≥ 60 s / ≥ 5 min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1b-1: L1 never ran, Wazuh still alerted ~1 min after first read; bucket public 6 min 25 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep rules always on; canary test after changes; alert if 100101 not followed by an L1 confirmation within 2 min</t>
+  </si>
+  <si>
     <t xml:space="preserve">Phase 5</t>
   </si>
   <si>
-    <t xml:space="preserve">In progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.15, 5.23, 8.3, 8.12, 8.24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 Storage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long-lived CI access key leaked through source code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dev-ci IAM user, data bucket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">External attacker / secret-scanning bots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Static key stored in a file in Git history; no secret scanning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Least-privilege dev-ci (no kms:Decrypt); Wazuh 100110 (unknown IP); RB-S2 runbook</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Detected 3 min 41 s after first misuse; contained 2 min 42 s after alert; KMS copy denied</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OIDC federation for CI (no standing keys); pre-commit + push-protection secret scanning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recommended</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.17, 8.4, 8.5, 8.28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 IAM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attacker persistence through additional access keys</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IAM users</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attacker holding a valid key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identity allowed to create its own keys</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wazuh 100113 (level 14) via us-east-1 IAM poller; AWSDenyAll-first containment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Persistence detected 3 min 40 s after creation; neutralized 5 min 21 s after creation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remove iam:CreateAccessKey from CI identities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.16, 5.18, 8.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Administrative port exposed to the internet and attacked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EC2 web instance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internet scanners, brute force</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Security group can be opened to 0.0.0.0/0; no NACL second layer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No key pair, no password auth, SSM only; Wazuh 100121 + 5710/5712; Lambda L2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hydra aborted (no password auth); S3a manual 7 min 57 s; S3b L2 5.3 s; agent detection in seconds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restrictive NACL; VPC flow logs; 100121+57xx correlation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.20, 8.22, 8.5, 8.16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 Networking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Instance role credentials stolen through IMDSv1 + SSRF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M-IMDS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lab-web-role credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attacker exploiting a web SSRF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMDSv1 can be re-enabled per instance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMDSv2 required, hop limit 1; Lambda L3; Wazuh 100132; rules 100130/131/133 for credential use outside the instance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L3 fixed in 6.4 s; 100132 in 1 min 23 s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Account default IMDSv2 (modify-instance-metadata-defaults)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.9, 8.20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automated remediation silently not working</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S1b-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lambda L1-L3 / EventBridge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational failure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rule changes and new trails are eventually consistent; no health check of automation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIEM detection independent of automation; session checklist (wait ≥ 60 s / ≥ 5 min)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S1b-1: L1 never ran, Wazuh still alerted ~1 min after first read; bucket public 6 min 25 s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keep rules always on; canary test after changes; alert if 100101 not followed by an L1 confirmation within 2 min</t>
-  </si>
-  <si>
     <t xml:space="preserve">8.16, 5.30</t>
   </si>
   <si>
@@ -369,9 +372,6 @@
     <t xml:space="preserve">Done</t>
   </si>
   <si>
-    <t xml:space="preserve">Closed</t>
-  </si>
-  <si>
     <t xml:space="preserve">R09</t>
   </si>
   <si>
@@ -417,13 +417,16 @@
     <t xml:space="preserve">AdministratorAccess on a user with a CLI key</t>
   </si>
   <si>
-    <t xml:space="preserve">MFA on console, key only on the laptop, budget alert, own-admin activity logged (100143)</t>
+    <t xml:space="preserve">MFA on console, key only on the laptop, budget alert, own-admin activity logged (100143), password policy (CIS 2.8/2.9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardening attempt showed groups are denied by the account SCP</t>
   </si>
   <si>
     <t xml:space="preserve">Accept (temporary)</t>
   </si>
   <si>
-    <t xml:space="preserve">Move policy to an admins group (Phase 5); delete the key at Phase 6</t>
+    <t xml:space="preserve">Groups blocked by an AWS-managed SCP (explicit deny on iam:CreateGroup, 2026-10-25); delete the key at Phase 6</t>
   </si>
   <si>
     <t xml:space="preserve">Phase 6</t>
@@ -1744,36 +1747,36 @@
         <v>33</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="U7" s="3" t="s">
         <v>48</v>
       </c>
       <c r="V7" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W7" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>4</v>
@@ -1790,10 +1793,10 @@
         <v>High</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>2</v>
@@ -1810,45 +1813,45 @@
         <v>Low</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="S8" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U8" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>4</v>
@@ -1865,10 +1868,10 @@
         <v>High</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>1</v>
@@ -1888,22 +1891,22 @@
         <v>31</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="S9" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="U9" s="3" t="s">
-        <v>114</v>
+        <v>35</v>
       </c>
       <c r="V9" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="W9" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1943,7 +1946,7 @@
         <v>121</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>2</v>
@@ -1969,19 +1972,19 @@
         <v>33</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U10" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="V10" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>124</v>
       </c>
@@ -2018,7 +2021,7 @@
         <v>130</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>2</v>
@@ -2035,22 +2038,22 @@
         <v>Medium</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="S11" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="U11" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="V11" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="W11" s="2" t="s">
         <v>50</v>
@@ -2058,22 +2061,22 @@
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>2</v>
@@ -2090,10 +2093,10 @@
         <v>Low</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>2</v>
@@ -2110,45 +2113,45 @@
         <v>Low</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="S12" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="U12" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="W12" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="V12" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="W12" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>117</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>2</v>
@@ -2165,10 +2168,10 @@
         <v>Medium</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>2</v>
@@ -2188,42 +2191,42 @@
         <v>31</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="S13" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="U13" s="3" t="s">
         <v>48</v>
       </c>
       <c r="V13" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="W13" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>4</v>
@@ -2240,10 +2243,10 @@
         <v>Medium</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>3</v>
@@ -2263,42 +2266,42 @@
         <v>122</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="S14" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U14" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="V14" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="W14" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="V14" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="W14" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>118</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>4</v>
@@ -2315,10 +2318,10 @@
         <v>Medium</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>3</v>
@@ -2335,45 +2338,45 @@
         <v>Low</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S15" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U15" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="V15" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="W15" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>3</v>
@@ -2390,10 +2393,10 @@
         <v>Medium</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>1</v>
@@ -2413,42 +2416,42 @@
         <v>31</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="S16" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="U16" s="3" t="s">
-        <v>114</v>
+        <v>35</v>
       </c>
       <c r="V16" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="W16" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>4</v>
@@ -2465,10 +2468,10 @@
         <v>High</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>3</v>
@@ -2488,42 +2491,42 @@
         <v>31</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="S17" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="U17" s="3" t="s">
         <v>48</v>
       </c>
       <c r="V17" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="W17" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>117</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>3</v>
@@ -2540,10 +2543,10 @@
         <v>Medium</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>2</v>
@@ -2563,22 +2566,22 @@
         <v>122</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="S18" s="2" t="s">
         <v>33</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U18" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="V18" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="W18" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="V18" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="W18" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -2640,20 +2643,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">COUNTIF('Risk register'!J2:J18,"High")</f>
@@ -2666,7 +2669,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">COUNTIF('Risk register'!J2:J18,"Medium")</f>
@@ -2679,7 +2682,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">COUNTIF('Risk register'!J2:J18,"Low")</f>
@@ -2692,7 +2695,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">COUNTA('Risk register'!A2:A18)</f>
@@ -2701,7 +2704,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">ROUND(AVERAGE('Risk register'!I2:I18),1)</f>
@@ -2714,7 +2717,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">COUNTIF('Risk register'!U2:U18,"Open")</f>
@@ -2723,16 +2726,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">COUNTIF('Risk register'!U2:U18,"In progress")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">COUNTIF('Risk register'!U2:U18,"Accepted")</f>
@@ -2741,11 +2744,11 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">COUNTIF('Risk register'!U2:U18,"Closed")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2773,42 +2776,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2816,23 +2819,23 @@
         <v>16</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>